<commit_message>
Etiketka shablonlari, Excel'da har qator alohida tovar, telefon ko'rinishi
- Etiketka shablonlari: o'lcham (mm), format, maydonlar tartibi, shrift, sinov chop etish
- Soni: kirim bo'yicha, qoldiq bo'yicha yoki har biriga 1
- Excel shablondan 'Necha pachka keldi' olib tashlandi; har qator alohida tovar
- Chek oynasi tugmalari tuzatildi; telefonda oynalar pastdan chiqadi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wy5ERXDjwmq7jHn5RV6tgD
</commit_message>
<xml_diff>
--- a/docs/tovarlar-shablon.xlsx
+++ b/docs/tovarlar-shablon.xlsx
@@ -29,9 +29,6 @@
   </si>
   <si>
     <t>Pachkada (juft)</t>
-  </si>
-  <si>
-    <t>Necha pachka keldi</t>
   </si>
   <si>
     <t>Kelish narxi (1 juft)</t>
@@ -107,9 +104,8 @@
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -134,33 +130,27 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>10</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
       </c>
       <c r="E2">
         <v>5</v>
       </c>
       <c r="F2">
-        <v>20</v>
+        <v>160000</v>
       </c>
       <c r="G2">
-        <v>160000</v>
-      </c>
-      <c r="H2">
         <v>190000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Tovar kodi: brend harfi + raqam (A1…A200), brendlar ro'yxati
- Har brendga harf; 200 dan keyin keyingi bo'sh harf
- Kod = shtrix-kod (CODE128): vitrina, etiketka va skanerda bir xil
- Sozlamalar → Brendlar: qo'shish, nomini o'zgartirish, keyingi kodni ko'rish
- Yangi tovar: brend ro'yxatdan, kod oldindan ko'rinadi, qo'lda kod (band bo'lsa xato)
- Excel: ixtiyoriy 'Kod' ustuni, takror va band kodlar tekshiriladi
- Skaner qisqa kodlarni ham taniydi; ruscha klaviaturadagi kod to'g'rilanadi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wy5ERXDjwmq7jHn5RV6tgD
</commit_message>
<xml_diff>
--- a/docs/tovarlar-shablon.xlsx
+++ b/docs/tovarlar-shablon.xlsx
@@ -15,6 +15,9 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <si>
+    <t>Kod (ixtiyoriy)</t>
+  </si>
   <si>
     <t>Brend</t>
   </si>
@@ -100,12 +103,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -130,11 +134,11 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
@@ -144,13 +148,16 @@
       <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2">
         <v>5</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>160000</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>190000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "Tovar kodi: brend harfi + raqam (A1…A200), brendlar ro'yxati"
This reverts commit 10c01fbdfa0484a2c45f45800cb2e4a5ad0fe9d7.
</commit_message>
<xml_diff>
--- a/docs/tovarlar-shablon.xlsx
+++ b/docs/tovarlar-shablon.xlsx
@@ -15,9 +15,6 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <si>
-    <t>Kod (ixtiyoriy)</t>
-  </si>
   <si>
     <t>Brend</t>
   </si>
@@ -103,13 +100,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -134,11 +130,11 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2">
       <c r="B2" t="s">
         <v>8</v>
       </c>
@@ -148,16 +144,13 @@
       <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
-        <v>11</v>
+      <c r="E2">
+        <v>5</v>
       </c>
       <c r="F2">
-        <v>5</v>
+        <v>160000</v>
       </c>
       <c r="G2">
-        <v>160000</v>
-      </c>
-      <c r="H2">
         <v>190000</v>
       </c>
     </row>

</xml_diff>